<commit_message>
Update resource import example for he
</commit_message>
<xml_diff>
--- a/public/example-files/resources_import_he.xlsx
+++ b/public/example-files/resources_import_he.xlsx
@@ -81,11 +81,6 @@
       <name val="Helvetica Neue"/>
     </font>
     <font>
-      <sz val="9"/>
-      <color indexed="8"/>
-      <name val="Arial"/>
-    </font>
-    <font>
       <sz val="15"/>
       <color indexed="8"/>
       <name val="Calibri"/>
@@ -95,6 +90,11 @@
       <sz val="9"/>
       <color indexed="8"/>
       <name val="&quot;Helvetica Neue&quot;"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="8"/>
+      <name val="Arial"/>
     </font>
     <font>
       <sz val="9"/>
@@ -134,7 +134,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor indexed="15"/>
+        <fgColor indexed="16"/>
         <bgColor auto="1"/>
       </patternFill>
     </fill>
@@ -145,7 +145,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="22">
+  <borders count="27">
     <border>
       <left/>
       <right/>
@@ -290,28 +290,13 @@
     </border>
     <border>
       <left style="thin">
-        <color indexed="10"/>
-      </left>
-      <right style="thin">
+        <color indexed="14"/>
+      </left>
+      <right style="thin">
+        <color indexed="14"/>
+      </right>
+      <top style="thin">
         <color indexed="13"/>
-      </right>
-      <top style="thin">
-        <color indexed="10"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="13"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="14"/>
-      </left>
-      <right style="thin">
-        <color indexed="14"/>
-      </right>
-      <top style="thin">
-        <color indexed="13"/>
       </top>
       <bottom style="thin">
         <color indexed="14"/>
@@ -365,13 +350,87 @@
     </border>
     <border>
       <left style="thin">
-        <color indexed="16"/>
-      </left>
-      <right style="thin">
-        <color indexed="16"/>
-      </right>
-      <top style="thin">
-        <color indexed="16"/>
+        <color indexed="14"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="14"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="14"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="14"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="14"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="14"/>
+      </right>
+      <top style="thin">
+        <color indexed="14"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="14"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="14"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="14"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="15"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="14"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="15"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="14"/>
+      </right>
+      <top style="thin">
+        <color indexed="14"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="15"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="15"/>
+      </left>
+      <right style="thin">
+        <color indexed="15"/>
+      </right>
+      <top style="thin">
+        <color indexed="15"/>
       </top>
       <bottom style="thin">
         <color indexed="17"/>
@@ -380,7 +439,7 @@
     </border>
     <border>
       <left style="thin">
-        <color indexed="16"/>
+        <color indexed="15"/>
       </left>
       <right style="thin">
         <color indexed="17"/>
@@ -389,7 +448,7 @@
         <color indexed="17"/>
       </top>
       <bottom style="thin">
-        <color indexed="16"/>
+        <color indexed="15"/>
       </bottom>
       <diagonal/>
     </border>
@@ -398,43 +457,43 @@
         <color indexed="17"/>
       </left>
       <right style="thin">
-        <color indexed="16"/>
+        <color indexed="15"/>
       </right>
       <top style="thin">
         <color indexed="17"/>
       </top>
       <bottom style="thin">
-        <color indexed="16"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="16"/>
-      </left>
-      <right style="thin">
-        <color indexed="16"/>
+        <color indexed="15"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="15"/>
+      </left>
+      <right style="thin">
+        <color indexed="15"/>
       </right>
       <top style="thin">
         <color indexed="17"/>
       </top>
       <bottom style="thin">
-        <color indexed="16"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="16"/>
+        <color indexed="15"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="15"/>
       </left>
       <right style="thin">
         <color indexed="17"/>
       </right>
       <top style="thin">
-        <color indexed="16"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="16"/>
+        <color indexed="15"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="15"/>
       </bottom>
       <diagonal/>
     </border>
@@ -443,28 +502,28 @@
         <color indexed="17"/>
       </left>
       <right style="thin">
-        <color indexed="16"/>
-      </right>
-      <top style="thin">
-        <color indexed="16"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="16"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="16"/>
-      </left>
-      <right style="thin">
-        <color indexed="16"/>
-      </right>
-      <top style="thin">
-        <color indexed="16"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="16"/>
+        <color indexed="15"/>
+      </right>
+      <top style="thin">
+        <color indexed="15"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="15"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="15"/>
+      </left>
+      <right style="thin">
+        <color indexed="15"/>
+      </right>
+      <top style="thin">
+        <color indexed="15"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="15"/>
       </bottom>
       <diagonal/>
     </border>
@@ -474,80 +533,95 @@
       <alignment vertical="bottom"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="2" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="3" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment horizontal="right" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment horizontal="right" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment horizontal="right" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment horizontal="right" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="3" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="5" fillId="3" borderId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="3" borderId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="4" fillId="3" borderId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment horizontal="right" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="3" borderId="8" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="3" borderId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="3" borderId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment horizontal="right" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="10" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="3" borderId="8" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="3" borderId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="3" borderId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="11" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="11" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="12" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="12" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="13" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="13" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="14" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="14" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="15" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="16" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="6" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="6" fillId="3" borderId="17" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="15" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="18" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="19" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="20" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="16" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="21" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="17" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="22" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="18" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="23" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="19" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="24" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="20" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="25" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="21" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="26" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
   </cellXfs>
@@ -573,8 +647,8 @@
       <rgbColor rgb="ffffffff"/>
       <rgbColor rgb="ff9a9a9a"/>
       <rgbColor rgb="ffaaaaaa"/>
+      <rgbColor rgb="ffa5a5a5"/>
       <rgbColor rgb="ffbdc0bf"/>
-      <rgbColor rgb="ffa5a5a5"/>
       <rgbColor rgb="ff3f3f3f"/>
       <rgbColor rgb="ffdbdbdb"/>
     </indexedColors>
@@ -1608,17 +1682,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr defaultColWidth="12.6667" defaultRowHeight="12.3" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="23.9688" style="1" customWidth="1"/>
-    <col min="2" max="2" width="19.7344" style="1" customWidth="1"/>
-    <col min="3" max="3" width="16.1016" style="1" customWidth="1"/>
-    <col min="4" max="4" width="21.375" style="1" customWidth="1"/>
+    <col min="1" max="1" width="24" style="1" customWidth="1"/>
+    <col min="2" max="2" width="19.8516" style="1" customWidth="1"/>
+    <col min="3" max="3" width="16.1719" style="1" customWidth="1"/>
+    <col min="4" max="4" width="21.3516" style="1" customWidth="1"/>
     <col min="5" max="5" width="17.5" style="1" customWidth="1"/>
-    <col min="6" max="6" width="22.5781" style="1" customWidth="1"/>
+    <col min="6" max="6" width="22.6719" style="1" customWidth="1"/>
     <col min="7" max="7" width="19.3516" style="1" customWidth="1"/>
-    <col min="8" max="8" width="9.71875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="9.67188" style="1" customWidth="1"/>
     <col min="9" max="16384" width="12.6719" style="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1667,7 +1741,7 @@
       <c r="F2" t="s" s="10">
         <v>13</v>
       </c>
-      <c r="G2" t="s" s="7">
+      <c r="G2" t="s" s="11">
         <v>12</v>
       </c>
       <c r="H2" t="s" s="11">
@@ -1682,7 +1756,7 @@
       <c r="E3" s="14"/>
       <c r="F3" s="14"/>
       <c r="G3" s="13"/>
-      <c r="H3" s="12"/>
+      <c r="H3" s="13"/>
     </row>
     <row r="4" ht="21.45" customHeight="1">
       <c r="A4" s="15"/>
@@ -1744,7 +1818,22 @@
       <c r="G9" s="15"/>
       <c r="H9" s="15"/>
     </row>
+    <row r="10" ht="13.65" customHeight="1">
+      <c r="A10" s="16"/>
+      <c r="B10" s="17"/>
+      <c r="C10" s="17"/>
+      <c r="D10" s="17"/>
+      <c r="E10" s="17"/>
+      <c r="F10" s="17"/>
+      <c r="G10" s="17"/>
+      <c r="H10" s="18"/>
+    </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2">
+      <formula1>"רפואי,בית,ילדים,רגשי,מיצוי זכויות,כללי"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="100" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>
   <headerFooter>
@@ -1758,91 +1847,91 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:E11"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr defaultColWidth="16.3333" defaultRowHeight="13.45" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="5" width="16.3516" style="16" customWidth="1"/>
-    <col min="6" max="16384" width="16.3516" style="16" customWidth="1"/>
+    <col min="1" max="5" width="16.3516" style="19" customWidth="1"/>
+    <col min="6" max="16384" width="16.3516" style="19" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="15.55" customHeight="1">
-      <c r="A1" t="s" s="17">
+      <c r="A1" t="s" s="20">
         <v>15</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="22"/>
     </row>
     <row r="2" ht="13.2" customHeight="1">
-      <c r="A2" s="18"/>
-      <c r="B2" s="18"/>
-      <c r="C2" s="18"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
+      <c r="A2" s="23"/>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
     </row>
     <row r="3" ht="13.2" customHeight="1">
-      <c r="A3" s="19"/>
-      <c r="B3" s="20"/>
-      <c r="C3" s="21"/>
-      <c r="D3" s="21"/>
-      <c r="E3" s="21"/>
+      <c r="A3" s="24"/>
+      <c r="B3" s="25"/>
+      <c r="C3" s="26"/>
+      <c r="D3" s="26"/>
+      <c r="E3" s="26"/>
     </row>
     <row r="4" ht="13" customHeight="1">
-      <c r="A4" s="22"/>
-      <c r="B4" s="23"/>
-      <c r="C4" s="24"/>
-      <c r="D4" s="24"/>
-      <c r="E4" s="24"/>
+      <c r="A4" s="27"/>
+      <c r="B4" s="28"/>
+      <c r="C4" s="29"/>
+      <c r="D4" s="29"/>
+      <c r="E4" s="29"/>
     </row>
     <row r="5" ht="13" customHeight="1">
-      <c r="A5" s="22"/>
-      <c r="B5" s="23"/>
-      <c r="C5" s="24"/>
-      <c r="D5" s="24"/>
-      <c r="E5" s="24"/>
+      <c r="A5" s="27"/>
+      <c r="B5" s="28"/>
+      <c r="C5" s="29"/>
+      <c r="D5" s="29"/>
+      <c r="E5" s="29"/>
     </row>
     <row r="6" ht="13" customHeight="1">
-      <c r="A6" s="22"/>
-      <c r="B6" s="23"/>
-      <c r="C6" s="24"/>
-      <c r="D6" s="24"/>
-      <c r="E6" s="24"/>
+      <c r="A6" s="27"/>
+      <c r="B6" s="28"/>
+      <c r="C6" s="29"/>
+      <c r="D6" s="29"/>
+      <c r="E6" s="29"/>
     </row>
     <row r="7" ht="13" customHeight="1">
-      <c r="A7" s="22"/>
-      <c r="B7" s="23"/>
-      <c r="C7" s="24"/>
-      <c r="D7" s="24"/>
-      <c r="E7" s="24"/>
+      <c r="A7" s="27"/>
+      <c r="B7" s="28"/>
+      <c r="C7" s="29"/>
+      <c r="D7" s="29"/>
+      <c r="E7" s="29"/>
     </row>
     <row r="8" ht="13" customHeight="1">
-      <c r="A8" s="22"/>
-      <c r="B8" s="23"/>
-      <c r="C8" s="24"/>
-      <c r="D8" s="24"/>
-      <c r="E8" s="24"/>
+      <c r="A8" s="27"/>
+      <c r="B8" s="28"/>
+      <c r="C8" s="29"/>
+      <c r="D8" s="29"/>
+      <c r="E8" s="29"/>
     </row>
     <row r="9" ht="13" customHeight="1">
-      <c r="A9" s="22"/>
-      <c r="B9" s="23"/>
-      <c r="C9" s="24"/>
-      <c r="D9" s="24"/>
-      <c r="E9" s="24"/>
+      <c r="A9" s="27"/>
+      <c r="B9" s="28"/>
+      <c r="C9" s="29"/>
+      <c r="D9" s="29"/>
+      <c r="E9" s="29"/>
     </row>
     <row r="10" ht="13" customHeight="1">
-      <c r="A10" s="22"/>
-      <c r="B10" s="23"/>
-      <c r="C10" s="24"/>
-      <c r="D10" s="24"/>
-      <c r="E10" s="24"/>
+      <c r="A10" s="27"/>
+      <c r="B10" s="28"/>
+      <c r="C10" s="29"/>
+      <c r="D10" s="29"/>
+      <c r="E10" s="29"/>
     </row>
     <row r="11" ht="13" customHeight="1">
-      <c r="A11" s="22"/>
-      <c r="B11" s="23"/>
-      <c r="C11" s="24"/>
-      <c r="D11" s="24"/>
-      <c r="E11" s="24"/>
+      <c r="A11" s="27"/>
+      <c r="B11" s="28"/>
+      <c r="C11" s="29"/>
+      <c r="D11" s="29"/>
+      <c r="E11" s="29"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>